<commit_message>
Remove local SQLite database and transition entirely to Supabase
</commit_message>
<xml_diff>
--- a/Synapse_Teams_Problem_Statements.xlsx
+++ b/Synapse_Teams_Problem_Statements.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b9506d999bd99790/Desktop/Ragav Folder/Projects/Hackthon site/Hackthon site/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="11_92AE971A298F49377C908C3A0036A9F5602AC939" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B8BCA2BE-3B75-45BB-9975-0679AB8E88FD}"/>
+  <xr:revisionPtr revIDLastSave="14" documentId="11_92AE971A298F49377C908C3A0036A9F5602AC939" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DDB5856D-37B1-4200-9301-E67AC8BB30B0}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Teams &amp; Problem Statements" sheetId="1" r:id="rId1"/>
     <sheet name="Paired Allocations" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Teams &amp; Problem Statements'!$A$1:$K$56</definedName>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="840" uniqueCount="400">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="946" uniqueCount="455">
   <si>
     <t>Team ID</t>
   </si>
@@ -1224,13 +1225,1240 @@
   </si>
   <si>
     <t>Pair 27</t>
+  </si>
+  <si>
+    <t>PS #</t>
+  </si>
+  <si>
+    <t>Assigned Teams</t>
+  </si>
+  <si>
+    <r>
+      <t>SY24</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> &amp; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10.8"/>
+        <color rgb="FFD0D0D0"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>SY50</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>⚔️ </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10.8"/>
+        <color rgb="FFD0D0D0"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>SY26</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> &amp; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10.8"/>
+        <color rgb="FFD0D0D0"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>SY52</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>(4 teams)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>SY04</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> &amp; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10.8"/>
+        <color rgb="FFD0D0D0"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>SY30</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>(2 teams)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>SY18</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> &amp; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10.8"/>
+        <color rgb="FFD0D0D0"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>SY44</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>(2 teams)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>SY06</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> &amp; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10.8"/>
+        <color rgb="FFD0D0D0"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>SY32</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>(2 teams)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>SY02</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> &amp; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10.8"/>
+        <color rgb="FFD0D0D0"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>SY28</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>(2 teams)</t>
+    </r>
+  </si>
+  <si>
+    <t>Automated Underwriting</t>
+  </si>
+  <si>
+    <r>
+      <t>SY23</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> &amp; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10.8"/>
+        <color rgb="FFD0D0D0"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>SY49</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>(2 teams)</t>
+    </r>
+  </si>
+  <si>
+    <t>InsurTech Claims</t>
+  </si>
+  <si>
+    <r>
+      <t>SY17</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> &amp; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10.8"/>
+        <color rgb="FFD0D0D0"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>SY43</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>(2 teams)</t>
+    </r>
+  </si>
+  <si>
+    <t>InsurTech &amp; Telematics</t>
+  </si>
+  <si>
+    <r>
+      <t>SY07</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> &amp; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10.8"/>
+        <color rgb="FFD0D0D0"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>SY33</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>(2 teams)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>SY14</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> &amp; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10.8"/>
+        <color rgb="FFD0D0D0"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>SY40</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>(2 teams)</t>
+    </r>
+  </si>
+  <si>
+    <t>ClimateTech &amp; Risk</t>
+  </si>
+  <si>
+    <r>
+      <t>SY01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> &amp; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10.8"/>
+        <color rgb="FFD0D0D0"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>SY27</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>(2 teams)</t>
+    </r>
+  </si>
+  <si>
+    <t>HealthTech</t>
+  </si>
+  <si>
+    <r>
+      <t>SY25</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> &amp; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10.8"/>
+        <color rgb="FFD0D0D0"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>SY51</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>(2 teams)</t>
+    </r>
+  </si>
+  <si>
+    <t>HealthTech Speech NLP</t>
+  </si>
+  <si>
+    <r>
+      <t>SY16</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> &amp; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10.8"/>
+        <color rgb="FFD0D0D0"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>SY42</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>(2 teams)</t>
+    </r>
+  </si>
+  <si>
+    <t>FHIR Interoperability</t>
+  </si>
+  <si>
+    <r>
+      <t>SY22</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> &amp; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10.8"/>
+        <color rgb="FFD0D0D0"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>SY48</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>(2 teams)</t>
+    </r>
+  </si>
+  <si>
+    <t>Predictive Health AI</t>
+  </si>
+  <si>
+    <r>
+      <t>SY13</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> &amp; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10.8"/>
+        <color rgb="FFD0D0D0"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>SY39</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>(2 teams)</t>
+    </r>
+  </si>
+  <si>
+    <t>HealthTech Analytics</t>
+  </si>
+  <si>
+    <r>
+      <t>SY19</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> &amp; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10.8"/>
+        <color rgb="FFD0D0D0"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>SY45</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>(2 teams)</t>
+    </r>
+  </si>
+  <si>
+    <t>Decentralized AI Agent Orchestrator</t>
+  </si>
+  <si>
+    <t>Disaster Response Mesh AI</t>
+  </si>
+  <si>
+    <r>
+      <t>SY20</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> &amp; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10.8"/>
+        <color rgb="FFD0D0D0"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>SY46</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>(2 teams)</t>
+    </r>
+  </si>
+  <si>
+    <t>Vision &amp; Accessibility</t>
+  </si>
+  <si>
+    <r>
+      <t>SY10</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> &amp; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10.8"/>
+        <color rgb="FFD0D0D0"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>SY36</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>(2 teams)</t>
+    </r>
+  </si>
+  <si>
+    <t>Enterprise Legal Intelligence &amp; Compliance</t>
+  </si>
+  <si>
+    <t>LegalTech Copilot</t>
+  </si>
+  <si>
+    <r>
+      <t>SY11</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> &amp; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10.8"/>
+        <color rgb="FFD0D0D0"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>SY37</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>(2 teams)</t>
+    </r>
+  </si>
+  <si>
+    <t>Enterprise Multi-Source RAG Intelligence</t>
+  </si>
+  <si>
+    <t>Enterprise RAG</t>
+  </si>
+  <si>
+    <r>
+      <t>SY05</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> &amp; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10.8"/>
+        <color rgb="FFD0D0D0"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>SY31</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>(2 teams)</t>
+    </r>
+  </si>
+  <si>
+    <t>AI Grievance Redressal System</t>
+  </si>
+  <si>
+    <t>GovTech NLP</t>
+  </si>
+  <si>
+    <r>
+      <t>SY15</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> &amp; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10.8"/>
+        <color rgb="FFD0D0D0"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>SY41</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>(2 teams)</t>
+    </r>
+  </si>
+  <si>
+    <t>Public Health Analytics</t>
+  </si>
+  <si>
+    <r>
+      <t>SY09</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> &amp; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10.8"/>
+        <color rgb="FFD0D0D0"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>SY35</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>(2 teams)</t>
+    </r>
+  </si>
+  <si>
+    <t>Supply Chain Provenance for Pharmaceuticals</t>
+  </si>
+  <si>
+    <t>Blockchain</t>
+  </si>
+  <si>
+    <r>
+      <t>SY12</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> &amp; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10.8"/>
+        <color rgb="FFD0D0D0"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>SY38</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>(2 teams)</t>
+    </r>
+  </si>
+  <si>
+    <t>AI Agent Defense</t>
+  </si>
+  <si>
+    <r>
+      <t>SY21</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> &amp; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10.8"/>
+        <color rgb="FFD0D0D0"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>SY47</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>(2 teams)</t>
+    </r>
+  </si>
+  <si>
+    <t>Digital Evidence Integrity &amp; Fraud Platform</t>
+  </si>
+  <si>
+    <t>Digital Forensics</t>
+  </si>
+  <si>
+    <r>
+      <t>SY03</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> &amp; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10.8"/>
+        <color rgb="FFD0D0D0"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>SY29</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>⚔️ </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10.8"/>
+        <color rgb="FFD0D0D0"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>SY53</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> &amp; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10.8"/>
+        <color rgb="FFD0D0D0"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>SY54</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>(4 teams)</t>
+    </r>
+  </si>
+  <si>
+    <t>Usage-Based Insurance (Smart Mobility)</t>
+  </si>
+  <si>
+    <t>Smart Mobility</t>
+  </si>
+  <si>
+    <r>
+      <t>SY08</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> &amp; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10.8"/>
+        <color rgb="FFD0D0D0"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>SY34</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>(2 teams)</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1238,8 +2466,41 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FFCCCCCC"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FFCCCCCC"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8"/>
+      <color rgb="FFCCCCCC"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10.8"/>
+      <color rgb="FFD0D0D0"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="8"/>
+      <color rgb="FFCCCCCC"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1252,8 +2513,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF181818"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -1276,14 +2543,161 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4357,4 +5771,408 @@
     <ignoredError sqref="A1:H28" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B418B3E9-051A-4566-BC47-19DE39DA0922}">
+  <dimension ref="A1:D28"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="4.796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.09765625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.19921875" customWidth="1"/>
+    <col min="4" max="4" width="28.19921875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="34.799999999999997" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="3" t="s">
+        <v>400</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A2" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="B2" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="C2" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="12"/>
+      <c r="B3" s="14"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="7" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="8" t="s">
+        <v>183</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>184</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>185</v>
+      </c>
+      <c r="D4" s="10" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="34.799999999999997" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="34.799999999999997" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="8" t="s">
+        <v>176</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>177</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>177</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>408</v>
+      </c>
+      <c r="D8" s="10" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="34.799999999999997" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="C9" s="9" t="s">
+        <v>410</v>
+      </c>
+      <c r="D9" s="10" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>145</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>412</v>
+      </c>
+      <c r="D10" s="10" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="34.799999999999997" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="8" t="s">
+        <v>207</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>208</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>209</v>
+      </c>
+      <c r="D11" s="10" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="34.799999999999997" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="B12" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>415</v>
+      </c>
+      <c r="D12" s="10" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="34.799999999999997" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="C13" s="9" t="s">
+        <v>417</v>
+      </c>
+      <c r="D13" s="10" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="34.799999999999997" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="C14" s="9" t="s">
+        <v>419</v>
+      </c>
+      <c r="D14" s="10" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="34.799999999999997" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="8" t="s">
+        <v>152</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="C15" s="9" t="s">
+        <v>421</v>
+      </c>
+      <c r="D15" s="10" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="8" t="s">
+        <v>160</v>
+      </c>
+      <c r="B16" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="C16" s="9" t="s">
+        <v>423</v>
+      </c>
+      <c r="D16" s="10" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="8" t="s">
+        <v>168</v>
+      </c>
+      <c r="B17" s="9" t="s">
+        <v>169</v>
+      </c>
+      <c r="C17" s="9" t="s">
+        <v>425</v>
+      </c>
+      <c r="D17" s="10" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="34.799999999999997" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="8" t="s">
+        <v>191</v>
+      </c>
+      <c r="B18" s="9" t="s">
+        <v>427</v>
+      </c>
+      <c r="C18" s="9" t="s">
+        <v>428</v>
+      </c>
+      <c r="D18" s="10" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="46.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="B19" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C19" s="9" t="s">
+        <v>430</v>
+      </c>
+      <c r="D19" s="10" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="46.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="B20" s="9" t="s">
+        <v>432</v>
+      </c>
+      <c r="C20" s="9" t="s">
+        <v>433</v>
+      </c>
+      <c r="D20" s="10" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="46.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="B21" s="9" t="s">
+        <v>435</v>
+      </c>
+      <c r="C21" s="9" t="s">
+        <v>436</v>
+      </c>
+      <c r="D21" s="10" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="34.799999999999997" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="8" t="s">
+        <v>128</v>
+      </c>
+      <c r="B22" s="9" t="s">
+        <v>438</v>
+      </c>
+      <c r="C22" s="9" t="s">
+        <v>439</v>
+      </c>
+      <c r="D22" s="10" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="57.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="8" t="s">
+        <v>136</v>
+      </c>
+      <c r="B23" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="C23" s="9" t="s">
+        <v>441</v>
+      </c>
+      <c r="D23" s="10" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="57.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="B24" s="9" t="s">
+        <v>443</v>
+      </c>
+      <c r="C24" s="9" t="s">
+        <v>444</v>
+      </c>
+      <c r="D24" s="10" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B25" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="C25" s="9" t="s">
+        <v>446</v>
+      </c>
+      <c r="D25" s="10" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A26" s="11" t="s">
+        <v>199</v>
+      </c>
+      <c r="B26" s="13" t="s">
+        <v>448</v>
+      </c>
+      <c r="C26" s="13" t="s">
+        <v>449</v>
+      </c>
+      <c r="D26" s="6" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" ht="40.799999999999997" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="12"/>
+      <c r="B27" s="14"/>
+      <c r="C27" s="14"/>
+      <c r="D27" s="7" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="46.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="8" t="s">
+        <v>215</v>
+      </c>
+      <c r="B28" s="9" t="s">
+        <v>452</v>
+      </c>
+      <c r="C28" s="9" t="s">
+        <v>453</v>
+      </c>
+      <c r="D28" s="10" t="s">
+        <v>454</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="A26:A27"/>
+    <mergeCell ref="B26:B27"/>
+    <mergeCell ref="C26:C27"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>